<commit_message>
Add: 2 new Char
</commit_message>
<xml_diff>
--- a/data/游戏配置表.xlsx
+++ b/data/游戏配置表.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="195">
   <si>
     <t>角色名称</t>
   </si>
@@ -136,6 +136,18 @@
     <t>xuemo</t>
   </si>
   <si>
+    <t>反伤者</t>
+  </si>
+  <si>
+    <t>fanshang</t>
+  </si>
+  <si>
+    <t>建造者</t>
+  </si>
+  <si>
+    <t>jianzao</t>
+  </si>
+  <si>
     <t>技能等级</t>
   </si>
   <si>
@@ -437,6 +449,84 @@
   </si>
   <si>
     <t>使用普通技能时摸牌张数</t>
+  </si>
+  <si>
+    <t>反弹下次攻击消耗的能量</t>
+  </si>
+  <si>
+    <t>技能免疫消耗的能量</t>
+  </si>
+  <si>
+    <t>使用强化技能需要的最低点数</t>
+  </si>
+  <si>
+    <t>强化免疫阶段数</t>
+  </si>
+  <si>
+    <t>技能免疫持续的阶段数</t>
+  </si>
+  <si>
+    <t>解放技能消耗</t>
+  </si>
+  <si>
+    <t>解放技能消耗的能量</t>
+  </si>
+  <si>
+    <t>解放技能点数阈值</t>
+  </si>
+  <si>
+    <t>触发解放需要的最低技能牌点数</t>
+  </si>
+  <si>
+    <t>解放免疫阶段数</t>
+  </si>
+  <si>
+    <t>全免疫+反弹持续的阶段数（约2回合）</t>
+  </si>
+  <si>
+    <t>工人基础效率</t>
+  </si>
+  <si>
+    <t>每个小人每阶段建造的进度（基础值）</t>
+  </si>
+  <si>
+    <t>一层房效率加成</t>
+  </si>
+  <si>
+    <t>超过1层房子时工人效率额外加成</t>
+  </si>
+  <si>
+    <t>二层房减伤</t>
+  </si>
+  <si>
+    <t>超过2层房子时受伤减免值</t>
+  </si>
+  <si>
+    <t>三层房回血</t>
+  </si>
+  <si>
+    <t>达到3层房子时每回合回血量</t>
+  </si>
+  <si>
+    <t>房子减半伤害阈值</t>
+  </si>
+  <si>
+    <t>单次伤害超过此值时房子减半</t>
+  </si>
+  <si>
+    <t>解放最低房子数</t>
+  </si>
+  <si>
+    <t>触发解放需要的最低房子层数</t>
+  </si>
+  <si>
+    <t>解放最低点数</t>
+  </si>
+  <si>
+    <t>解放最高点数</t>
+  </si>
+  <si>
+    <t>触发解放的最高技能牌点数</t>
   </si>
   <si>
     <t>场地名称</t>
@@ -1187,6 +1277,64 @@
         <v>19</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12">
+        <v>95</v>
+      </c>
+      <c r="D12">
+        <v>100</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12" t="s">
+        <v>34</v>
+      </c>
+      <c r="G12" t="s">
+        <v>19</v>
+      </c>
+      <c r="H12" t="s">
+        <v>19</v>
+      </c>
+      <c r="I12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13">
+        <v>90</v>
+      </c>
+      <c r="D13">
+        <v>100</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13" t="s">
+        <v>34</v>
+      </c>
+      <c r="G13" t="s">
+        <v>19</v>
+      </c>
+      <c r="H13" t="s">
+        <v>19</v>
+      </c>
+      <c r="I13" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -1207,42 +1355,42 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>11</v>
@@ -1263,7 +1411,7 @@
         <v>14</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3">
@@ -1271,10 +1419,10 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D3">
         <v>10</v>
@@ -1295,7 +1443,7 @@
         <v>19</v>
       </c>
       <c r="J3" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4">
@@ -1303,10 +1451,10 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D4">
         <v>20</v>
@@ -1327,7 +1475,7 @@
         <v>19</v>
       </c>
       <c r="J4" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5">
@@ -1335,10 +1483,10 @@
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="D5">
         <v>80</v>
@@ -1359,7 +1507,7 @@
         <v>19</v>
       </c>
       <c r="J5" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6">
@@ -1379,10 +1527,10 @@
         <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D7">
         <v>8</v>
@@ -1403,7 +1551,7 @@
         <v>19</v>
       </c>
       <c r="J7" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8">
@@ -1411,10 +1559,10 @@
         <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D8">
         <v>16</v>
@@ -1435,7 +1583,7 @@
         <v>19</v>
       </c>
       <c r="J8" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9">
@@ -1443,10 +1591,10 @@
         <v>20</v>
       </c>
       <c r="B9" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C9" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D9">
         <v>80</v>
@@ -1467,7 +1615,7 @@
         <v>19</v>
       </c>
       <c r="J9" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10">
@@ -1487,10 +1635,10 @@
         <v>22</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D11" s="4">
         <v>5</v>
@@ -1511,7 +1659,7 @@
         <v>19</v>
       </c>
       <c r="J11" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12">
@@ -1519,10 +1667,10 @@
         <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C12" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D12">
         <v>10</v>
@@ -1543,7 +1691,7 @@
         <v>19</v>
       </c>
       <c r="J12" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13">
@@ -1551,10 +1699,10 @@
         <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C13" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D13">
         <v>60</v>
@@ -1575,7 +1723,7 @@
         <v>19</v>
       </c>
       <c r="J13" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14">
@@ -1595,10 +1743,10 @@
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C15" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D15">
         <v>10</v>
@@ -1619,7 +1767,7 @@
         <v>19</v>
       </c>
       <c r="J15" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16">
@@ -1627,10 +1775,10 @@
         <v>24</v>
       </c>
       <c r="B16" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C16" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D16">
         <v>20</v>
@@ -1651,7 +1799,7 @@
         <v>19</v>
       </c>
       <c r="J16" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17">
@@ -1659,10 +1807,10 @@
         <v>24</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D17" s="4">
         <v>80</v>
@@ -1683,7 +1831,7 @@
         <v>19</v>
       </c>
       <c r="J17" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18">
@@ -1703,10 +1851,10 @@
         <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C19" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D19">
         <v>10</v>
@@ -1727,7 +1875,7 @@
         <v>19</v>
       </c>
       <c r="J19" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20">
@@ -1735,10 +1883,10 @@
         <v>26</v>
       </c>
       <c r="B20" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C20" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D20">
         <v>20</v>
@@ -1759,7 +1907,7 @@
         <v>19</v>
       </c>
       <c r="J20" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21">
@@ -1767,10 +1915,10 @@
         <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C21" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D21">
         <v>80</v>
@@ -1791,7 +1939,7 @@
         <v>19</v>
       </c>
       <c r="J21" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22">
@@ -1811,10 +1959,10 @@
         <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C23" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D23">
         <v>8</v>
@@ -1835,7 +1983,7 @@
         <v>19</v>
       </c>
       <c r="J23" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="24">
@@ -1843,10 +1991,10 @@
         <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C24" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="D24">
         <v>16</v>
@@ -1867,7 +2015,7 @@
         <v>19</v>
       </c>
       <c r="J24" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="25">
@@ -1875,10 +2023,10 @@
         <v>28</v>
       </c>
       <c r="B25" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C25" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D25">
         <v>0</v>
@@ -1899,7 +2047,7 @@
         <v>19</v>
       </c>
       <c r="J25" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="26">
@@ -1937,6 +2085,12 @@
       <c r="H28" s="4"/>
       <c r="I28" s="4"/>
       <c r="J28" s="4"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -1957,13 +2111,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2">
@@ -1971,13 +2125,13 @@
         <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C2" t="s">
         <v>31</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3">
@@ -1985,13 +2139,13 @@
         <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C3">
         <v>60</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4">
@@ -1999,13 +2153,13 @@
         <v>32</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C4">
         <v>60</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5">
@@ -2013,13 +2167,13 @@
         <v>32</v>
       </c>
       <c r="B5" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C5">
         <v>3</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6">
@@ -2027,13 +2181,13 @@
         <v>32</v>
       </c>
       <c r="B6" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C6">
         <v>2</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7">
@@ -2041,13 +2195,13 @@
         <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C7">
         <v>15</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8">
@@ -2055,13 +2209,13 @@
         <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C8">
         <v>30</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9">
@@ -2069,13 +2223,13 @@
         <v>32</v>
       </c>
       <c r="B9" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C9">
         <v>3</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10">
@@ -2083,13 +2237,13 @@
         <v>32</v>
       </c>
       <c r="B10" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C10">
         <v>100</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12">
@@ -2097,13 +2251,13 @@
         <v>35</v>
       </c>
       <c r="B12" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C12" t="s">
         <v>31</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13">
@@ -2111,13 +2265,13 @@
         <v>35</v>
       </c>
       <c r="B13" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C13" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="14">
@@ -2125,13 +2279,13 @@
         <v>35</v>
       </c>
       <c r="B14" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C14">
         <v>2</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="15">
@@ -2139,13 +2293,13 @@
         <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C15">
         <v>2</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16">
@@ -2153,13 +2307,13 @@
         <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C16">
         <v>2</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="18">
@@ -2167,13 +2321,13 @@
         <v>37</v>
       </c>
       <c r="B18" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C18">
         <v>50</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="19">
@@ -2181,13 +2335,13 @@
         <v>37</v>
       </c>
       <c r="B19" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C19">
         <v>3</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20">
@@ -2195,13 +2349,13 @@
         <v>37</v>
       </c>
       <c r="B20" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C20">
         <v>30</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="21">
@@ -2209,13 +2363,13 @@
         <v>37</v>
       </c>
       <c r="B21" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C21">
         <v>25</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="22">
@@ -2223,13 +2377,13 @@
         <v>37</v>
       </c>
       <c r="B22" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C22">
         <v>3</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="23">
@@ -2237,13 +2391,13 @@
         <v>37</v>
       </c>
       <c r="B23" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C23">
         <v>20</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
     </row>
     <row r="24">
@@ -2251,13 +2405,13 @@
         <v>37</v>
       </c>
       <c r="B24" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C24">
         <v>10</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="25">
@@ -2265,13 +2419,13 @@
         <v>37</v>
       </c>
       <c r="B25" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C25">
         <v>10</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="26">
@@ -2279,13 +2433,223 @@
         <v>37</v>
       </c>
       <c r="B26" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C26">
         <v>2</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>139</v>
+        <v>143</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>39</v>
+      </c>
+      <c r="B28" t="s">
+        <v>108</v>
+      </c>
+      <c r="C28">
+        <v>10</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>39</v>
+      </c>
+      <c r="B29" t="s">
+        <v>110</v>
+      </c>
+      <c r="C29">
+        <v>15</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>39</v>
+      </c>
+      <c r="B30" t="s">
+        <v>112</v>
+      </c>
+      <c r="C30">
+        <v>3</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>39</v>
+      </c>
+      <c r="B31" t="s">
+        <v>147</v>
+      </c>
+      <c r="C31">
+        <v>3</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32" t="s">
+        <v>149</v>
+      </c>
+      <c r="C32">
+        <v>50</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33" t="s">
+        <v>151</v>
+      </c>
+      <c r="C33">
+        <v>25</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>39</v>
+      </c>
+      <c r="B34" t="s">
+        <v>153</v>
+      </c>
+      <c r="C34">
+        <v>10</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>41</v>
+      </c>
+      <c r="B36" t="s">
+        <v>155</v>
+      </c>
+      <c r="C36">
+        <v>1</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>41</v>
+      </c>
+      <c r="B37" t="s">
+        <v>157</v>
+      </c>
+      <c r="C37">
+        <v>2</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>41</v>
+      </c>
+      <c r="B38" t="s">
+        <v>159</v>
+      </c>
+      <c r="C38">
+        <v>2</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" t="s">
+        <v>161</v>
+      </c>
+      <c r="C39">
+        <v>5</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>41</v>
+      </c>
+      <c r="B40" t="s">
+        <v>163</v>
+      </c>
+      <c r="C40">
+        <v>20</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>41</v>
+      </c>
+      <c r="B41" t="s">
+        <v>165</v>
+      </c>
+      <c r="C41">
+        <v>5</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>167</v>
+      </c>
+      <c r="C42">
+        <v>20</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>41</v>
+      </c>
+      <c r="B43" t="s">
+        <v>168</v>
+      </c>
+      <c r="C43">
+        <v>25</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -2302,28 +2666,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>170</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>141</v>
+        <v>171</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>142</v>
+        <v>172</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>143</v>
+        <v>173</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>144</v>
+        <v>174</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>145</v>
+        <v>175</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>146</v>
+        <v>176</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>147</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2">
@@ -2340,7 +2704,7 @@
         <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>148</v>
+        <v>178</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>15</v>
@@ -2354,10 +2718,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>149</v>
+        <v>179</v>
       </c>
       <c r="B3" t="s">
-        <v>150</v>
+        <v>180</v>
       </c>
       <c r="C3" t="s">
         <v>19</v>
@@ -2380,10 +2744,10 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>151</v>
+        <v>181</v>
       </c>
       <c r="B4" t="s">
-        <v>152</v>
+        <v>182</v>
       </c>
       <c r="C4" t="s">
         <v>31</v>
@@ -2406,10 +2770,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>153</v>
+        <v>183</v>
       </c>
       <c r="B5" t="s">
-        <v>154</v>
+        <v>184</v>
       </c>
       <c r="C5" t="s">
         <v>19</v>
@@ -2432,10 +2796,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>155</v>
+        <v>185</v>
       </c>
       <c r="B6" t="s">
-        <v>156</v>
+        <v>186</v>
       </c>
       <c r="C6" t="s">
         <v>19</v>
@@ -2458,10 +2822,10 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>157</v>
+        <v>187</v>
       </c>
       <c r="B7" t="s">
-        <v>158</v>
+        <v>188</v>
       </c>
       <c r="C7" t="s">
         <v>19</v>
@@ -2484,10 +2848,10 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>159</v>
+        <v>189</v>
       </c>
       <c r="B8" t="s">
-        <v>160</v>
+        <v>190</v>
       </c>
       <c r="C8" t="s">
         <v>19</v>
@@ -2510,10 +2874,10 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>161</v>
+        <v>191</v>
       </c>
       <c r="B9" t="s">
-        <v>162</v>
+        <v>192</v>
       </c>
       <c r="C9" t="s">
         <v>19</v>
@@ -2536,10 +2900,10 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>163</v>
+        <v>193</v>
       </c>
       <c r="B10" t="s">
-        <v>164</v>
+        <v>194</v>
       </c>
       <c r="C10" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
chore(data): regen 游戏配置表.xlsx from JSON (Phase 1.8 Excel sync)
Reverse-pipeline run after Phase 1.3 renamed 4 field effects to
poker-suit IDs (diamond_real/void, spade_real/void). The xlsx
now reflects the new identifiers + display names (方片之境·实/虚,
黑桃之境·实/虚) for downstream Excel-editing workflows.

Generated via: go run ./cmd/jsontoexcel
Result: 16 characters / 8 fields
</commit_message>
<xml_diff>
--- a/data/游戏配置表.xlsx
+++ b/data/游戏配置表.xlsx
@@ -703,28 +703,28 @@
     <t>clear</t>
   </si>
   <si>
-    <t>虚幻之境·实</t>
-  </si>
-  <si>
-    <t>illusion_real</t>
-  </si>
-  <si>
-    <t>虚幻之境·虚</t>
-  </si>
-  <si>
-    <t>illusion_void</t>
-  </si>
-  <si>
-    <t>轮回之境·实</t>
-  </si>
-  <si>
-    <t>reinc_base</t>
-  </si>
-  <si>
-    <t>轮回之境·虚</t>
-  </si>
-  <si>
-    <t>reinc_other</t>
+    <t>方片之境·实</t>
+  </si>
+  <si>
+    <t>diamond_real</t>
+  </si>
+  <si>
+    <t>方片之境·虚</t>
+  </si>
+  <si>
+    <t>diamond_void</t>
+  </si>
+  <si>
+    <t>黑桃之境·实</t>
+  </si>
+  <si>
+    <t>spade_real</t>
+  </si>
+  <si>
+    <t>黑桃之境·虚</t>
+  </si>
+  <si>
+    <t>spade_void</t>
   </si>
   <si>
     <t>混沌之域</t>

</xml_diff>

<commit_message>
chore(data): regen 游戏配置表.xlsx with rokka + suou (Phase 5 / final)
Result: 18 characters / 8 fields (was 16 / 8 after Phase 1.8).

Non-blocking warnings:
- suou's hooks_config keys (fill_base, skip_cleanup_bonus, revive_timeout_sec,
  revive_unsynth_draw, revive_synth_draw) are not yet mapped in
  internal/excelmap/params.go — Excel cell uses the English key as a
  placeholder. Add Chinese mappings there if Excel-side editing is needed.

All server tests pass; phases 1-4 complete.
</commit_message>
<xml_diff>
--- a/data/游戏配置表.xlsx
+++ b/data/游戏配置表.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="260">
   <si>
     <t>角色名称</t>
   </si>
@@ -175,6 +175,18 @@
     <t>yuuki</t>
   </si>
   <si>
+    <t>六華</t>
+  </si>
+  <si>
+    <t>rokka</t>
+  </si>
+  <si>
+    <t>蘇芳</t>
+  </si>
+  <si>
+    <t>suou</t>
+  </si>
+  <si>
     <t>技能等级</t>
   </si>
   <si>
@@ -668,6 +680,48 @@
   </si>
   <si>
     <t>四印解放后每回合非首次命中时附加的恢复量</t>
+  </si>
+  <si>
+    <t>adjacent_draw</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>hand_size_cap</t>
+  </si>
+  <si>
+    <t>lit_eyes_needed</t>
+  </si>
+  <si>
+    <t>other_damage</t>
+  </si>
+  <si>
+    <t>other_draw</t>
+  </si>
+  <si>
+    <t>triangle_draw</t>
+  </si>
+  <si>
+    <t>triangle_heal</t>
+  </si>
+  <si>
+    <t>fill_base</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>revive_synth_draw</t>
+  </si>
+  <si>
+    <t>revive_timeout_sec</t>
+  </si>
+  <si>
+    <t>revive_unsynth_draw</t>
+  </si>
+  <si>
+    <t>skip_cleanup_bonus</t>
   </si>
   <si>
     <t>场地名称</t>
@@ -1489,6 +1543,46 @@
         <v>33</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>52</v>
+      </c>
+      <c r="B19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19">
+        <v>100</v>
+      </c>
+      <c r="D19">
+        <v>100</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20">
+        <v>30</v>
+      </c>
+      <c r="D20">
+        <v>30</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -1509,42 +1603,42 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>11</v>
@@ -1565,7 +1659,7 @@
         <v>14</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3">
@@ -1573,10 +1667,10 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D3">
         <v>10</v>
@@ -1585,7 +1679,7 @@
         <v>8</v>
       </c>
       <c r="J3" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4">
@@ -1593,10 +1687,10 @@
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C4" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D4">
         <v>20</v>
@@ -1605,7 +1699,7 @@
         <v>16</v>
       </c>
       <c r="J4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5">
@@ -1613,10 +1707,10 @@
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D5">
         <v>80</v>
@@ -1628,7 +1722,7 @@
         <v>20</v>
       </c>
       <c r="J5" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6">
@@ -1648,10 +1742,10 @@
         <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C7" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D7">
         <v>8</v>
@@ -1663,7 +1757,7 @@
         <v>2</v>
       </c>
       <c r="J7" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8">
@@ -1671,10 +1765,10 @@
         <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C8" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="D8">
         <v>16</v>
@@ -1686,7 +1780,7 @@
         <v>3</v>
       </c>
       <c r="J8" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9">
@@ -1694,10 +1788,10 @@
         <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C9" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D9">
         <v>80</v>
@@ -1712,7 +1806,7 @@
         <v>2</v>
       </c>
       <c r="J9" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10">
@@ -1732,10 +1826,10 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C11" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D11">
         <v>5</v>
@@ -1744,7 +1838,7 @@
         <v>20</v>
       </c>
       <c r="J11" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12">
@@ -1752,10 +1846,10 @@
         <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C12" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D12">
         <v>10</v>
@@ -1767,7 +1861,7 @@
         <v>30</v>
       </c>
       <c r="J12" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="13">
@@ -1775,10 +1869,10 @@
         <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C13" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D13">
         <v>60</v>
@@ -1793,7 +1887,7 @@
         <v>20</v>
       </c>
       <c r="J13" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14">
@@ -1813,10 +1907,10 @@
         <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C15" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D15">
         <v>10</v>
@@ -1828,7 +1922,7 @@
         <v>6</v>
       </c>
       <c r="J15" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16">
@@ -1836,10 +1930,10 @@
         <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C16" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D16">
         <v>20</v>
@@ -1851,7 +1945,7 @@
         <v>10</v>
       </c>
       <c r="J16" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="17">
@@ -1859,10 +1953,10 @@
         <v>23</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C17" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D17">
         <v>80</v>
@@ -1874,7 +1968,7 @@
         <v>20</v>
       </c>
       <c r="J17" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="18">
@@ -1894,10 +1988,10 @@
         <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C19" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D19">
         <v>10</v>
@@ -1906,7 +2000,7 @@
         <v>10</v>
       </c>
       <c r="J19" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="20">
@@ -1914,10 +2008,10 @@
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C20" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D20">
         <v>20</v>
@@ -1926,7 +2020,7 @@
         <v>20</v>
       </c>
       <c r="J20" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="21">
@@ -1934,10 +2028,10 @@
         <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C21" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D21">
         <v>80</v>
@@ -1946,7 +2040,7 @@
         <v>40</v>
       </c>
       <c r="J21" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22">
@@ -1966,10 +2060,10 @@
         <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C23" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D23">
         <v>8</v>
@@ -1978,7 +2072,7 @@
         <v>10</v>
       </c>
       <c r="J23" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="24">
@@ -1986,10 +2080,10 @@
         <v>27</v>
       </c>
       <c r="B24" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C24" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D24">
         <v>16</v>
@@ -2001,7 +2095,7 @@
         <v>10</v>
       </c>
       <c r="J24" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="25">
@@ -2009,10 +2103,10 @@
         <v>27</v>
       </c>
       <c r="B25" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C25" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="F25">
         <v>30</v>
@@ -2021,7 +2115,7 @@
         <v>10</v>
       </c>
       <c r="J25" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -2043,13 +2137,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2">
@@ -2057,13 +2151,13 @@
         <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C2" t="s">
         <v>30</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3">
@@ -2071,13 +2165,13 @@
         <v>31</v>
       </c>
       <c r="B3" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C3" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4">
@@ -2085,13 +2179,13 @@
         <v>31</v>
       </c>
       <c r="B4" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C4" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5">
@@ -2099,13 +2193,13 @@
         <v>31</v>
       </c>
       <c r="B5" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C5" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6">
@@ -2113,13 +2207,13 @@
         <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C6" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7">
@@ -2127,13 +2221,13 @@
         <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C7" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8">
@@ -2141,13 +2235,13 @@
         <v>31</v>
       </c>
       <c r="B8" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C8" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9">
@@ -2155,13 +2249,13 @@
         <v>31</v>
       </c>
       <c r="B9" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C9" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10">
@@ -2169,13 +2263,13 @@
         <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C10" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11">
@@ -2189,13 +2283,13 @@
         <v>34</v>
       </c>
       <c r="B12" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C12" t="s">
         <v>30</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="13">
@@ -2203,13 +2297,13 @@
         <v>34</v>
       </c>
       <c r="B13" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C13" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14">
@@ -2217,13 +2311,13 @@
         <v>34</v>
       </c>
       <c r="B14" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C14" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="15">
@@ -2231,13 +2325,13 @@
         <v>34</v>
       </c>
       <c r="B15" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C15" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
     </row>
     <row r="16">
@@ -2245,13 +2339,13 @@
         <v>34</v>
       </c>
       <c r="B16" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C16" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="17">
@@ -2265,13 +2359,13 @@
         <v>36</v>
       </c>
       <c r="B18" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C18" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19">
@@ -2279,13 +2373,13 @@
         <v>36</v>
       </c>
       <c r="B19" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C19" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="20">
@@ -2293,13 +2387,13 @@
         <v>36</v>
       </c>
       <c r="B20" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C20" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="21">
@@ -2307,13 +2401,13 @@
         <v>36</v>
       </c>
       <c r="B21" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C21" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="22">
@@ -2321,13 +2415,13 @@
         <v>36</v>
       </c>
       <c r="B22" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C22" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="23">
@@ -2335,13 +2429,13 @@
         <v>36</v>
       </c>
       <c r="B23" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="C23" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="24">
@@ -2349,13 +2443,13 @@
         <v>36</v>
       </c>
       <c r="B24" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C24" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="25">
@@ -2363,13 +2457,13 @@
         <v>36</v>
       </c>
       <c r="B25" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C25" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
     </row>
     <row r="26">
@@ -2377,13 +2471,13 @@
         <v>36</v>
       </c>
       <c r="B26" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="C26" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
     </row>
     <row r="27">
@@ -2391,13 +2485,13 @@
         <v>36</v>
       </c>
       <c r="B27" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C27" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="28">
@@ -2405,13 +2499,13 @@
         <v>36</v>
       </c>
       <c r="B28" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C28" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
     </row>
     <row r="29">
@@ -2425,13 +2519,13 @@
         <v>38</v>
       </c>
       <c r="B30" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C30" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="31">
@@ -2439,13 +2533,13 @@
         <v>38</v>
       </c>
       <c r="B31" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C31" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="32">
@@ -2453,13 +2547,13 @@
         <v>38</v>
       </c>
       <c r="B32" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C32" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="33">
@@ -2467,13 +2561,13 @@
         <v>38</v>
       </c>
       <c r="B33" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="C33" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
     </row>
     <row r="34">
@@ -2481,13 +2575,13 @@
         <v>38</v>
       </c>
       <c r="B34" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="C34" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="35">
@@ -2495,13 +2589,13 @@
         <v>38</v>
       </c>
       <c r="B35" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C35" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
     <row r="36">
@@ -2509,13 +2603,13 @@
         <v>38</v>
       </c>
       <c r="B36" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="C36" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="37">
@@ -2523,13 +2617,13 @@
         <v>38</v>
       </c>
       <c r="B37" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="C37" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
     </row>
     <row r="38">
@@ -2543,13 +2637,13 @@
         <v>40</v>
       </c>
       <c r="B39" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C39" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="40">
@@ -2557,13 +2651,13 @@
         <v>40</v>
       </c>
       <c r="B40" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C40" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="41">
@@ -2571,13 +2665,13 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C41" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="42">
@@ -2585,13 +2679,13 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="C42" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
     </row>
     <row r="43">
@@ -2599,13 +2693,13 @@
         <v>40</v>
       </c>
       <c r="B43" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="C43" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="44">
@@ -2613,13 +2707,13 @@
         <v>40</v>
       </c>
       <c r="B44" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="C44" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
     </row>
     <row r="45">
@@ -2627,13 +2721,13 @@
         <v>40</v>
       </c>
       <c r="B45" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C45" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
     </row>
     <row r="46">
@@ -2641,13 +2735,13 @@
         <v>40</v>
       </c>
       <c r="B46" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="C46" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
     </row>
     <row r="47">
@@ -2655,13 +2749,13 @@
         <v>40</v>
       </c>
       <c r="B47" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C47" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
     </row>
     <row r="48">
@@ -2669,13 +2763,13 @@
         <v>40</v>
       </c>
       <c r="B48" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="C48" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
     </row>
     <row r="49">
@@ -2689,13 +2783,13 @@
         <v>42</v>
       </c>
       <c r="B50" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C50" t="s">
         <v>30</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="51">
@@ -2703,13 +2797,13 @@
         <v>42</v>
       </c>
       <c r="B51" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C51" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="52">
@@ -2717,13 +2811,13 @@
         <v>42</v>
       </c>
       <c r="B52" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C52" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
     </row>
     <row r="53">
@@ -2737,13 +2831,13 @@
         <v>44</v>
       </c>
       <c r="B54" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C54" t="s">
         <v>30</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="55">
@@ -2751,13 +2845,13 @@
         <v>44</v>
       </c>
       <c r="B55" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C55" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="56">
@@ -2765,13 +2859,13 @@
         <v>44</v>
       </c>
       <c r="B56" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C56" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
     </row>
     <row r="57">
@@ -2779,13 +2873,13 @@
         <v>44</v>
       </c>
       <c r="B57" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C57" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="58">
@@ -2793,13 +2887,13 @@
         <v>44</v>
       </c>
       <c r="B58" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C58" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
     </row>
     <row r="59">
@@ -2813,13 +2907,13 @@
         <v>46</v>
       </c>
       <c r="B60" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C60" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
     </row>
     <row r="61">
@@ -2827,13 +2921,13 @@
         <v>46</v>
       </c>
       <c r="B61" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C61" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
     </row>
     <row r="62">
@@ -2841,13 +2935,13 @@
         <v>46</v>
       </c>
       <c r="B62" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C62" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
     </row>
     <row r="63">
@@ -2855,13 +2949,13 @@
         <v>46</v>
       </c>
       <c r="B63" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C63" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
     </row>
     <row r="64">
@@ -2869,13 +2963,13 @@
         <v>46</v>
       </c>
       <c r="B64" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C64" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="65">
@@ -2889,13 +2983,13 @@
         <v>48</v>
       </c>
       <c r="B66" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="C66" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="67">
@@ -2909,13 +3003,13 @@
         <v>50</v>
       </c>
       <c r="B68" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="C68" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
     </row>
     <row r="69">
@@ -2923,14 +3017,170 @@
         <v>50</v>
       </c>
       <c r="B69" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C69" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>216</v>
-      </c>
+        <v>220</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3"/>
+      <c r="B70" s="3"/>
+      <c r="C70" s="3"/>
+      <c r="D70" s="3"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="s">
+        <v>52</v>
+      </c>
+      <c r="B71" t="s">
+        <v>221</v>
+      </c>
+      <c r="C71" t="s">
+        <v>222</v>
+      </c>
+      <c r="D71" s="4"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
+        <v>52</v>
+      </c>
+      <c r="B72" t="s">
+        <v>223</v>
+      </c>
+      <c r="C72" t="s">
+        <v>125</v>
+      </c>
+      <c r="D72" s="4"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="s">
+        <v>52</v>
+      </c>
+      <c r="B73" t="s">
+        <v>224</v>
+      </c>
+      <c r="C73" t="s">
+        <v>119</v>
+      </c>
+      <c r="D73" s="4"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="s">
+        <v>52</v>
+      </c>
+      <c r="B74" t="s">
+        <v>225</v>
+      </c>
+      <c r="C74" t="s">
+        <v>168</v>
+      </c>
+      <c r="D74" s="4"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="s">
+        <v>52</v>
+      </c>
+      <c r="B75" t="s">
+        <v>226</v>
+      </c>
+      <c r="C75" t="s">
+        <v>168</v>
+      </c>
+      <c r="D75" s="4"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="s">
+        <v>52</v>
+      </c>
+      <c r="B76" t="s">
+        <v>227</v>
+      </c>
+      <c r="C76" t="s">
+        <v>119</v>
+      </c>
+      <c r="D76" s="4"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="s">
+        <v>52</v>
+      </c>
+      <c r="B77" t="s">
+        <v>228</v>
+      </c>
+      <c r="C77" t="s">
+        <v>168</v>
+      </c>
+      <c r="D77" s="4"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="3"/>
+      <c r="B78" s="3"/>
+      <c r="C78" s="3"/>
+      <c r="D78" s="3"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="s">
+        <v>54</v>
+      </c>
+      <c r="B79" t="s">
+        <v>229</v>
+      </c>
+      <c r="C79" t="s">
+        <v>230</v>
+      </c>
+      <c r="D79" s="4"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="s">
+        <v>54</v>
+      </c>
+      <c r="B80" t="s">
+        <v>231</v>
+      </c>
+      <c r="C80" t="s">
+        <v>222</v>
+      </c>
+      <c r="D80" s="4"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="s">
+        <v>54</v>
+      </c>
+      <c r="B81" t="s">
+        <v>232</v>
+      </c>
+      <c r="C81" t="s">
+        <v>125</v>
+      </c>
+      <c r="D81" s="4"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="s">
+        <v>54</v>
+      </c>
+      <c r="B82" t="s">
+        <v>233</v>
+      </c>
+      <c r="C82" t="s">
+        <v>230</v>
+      </c>
+      <c r="D82" s="4"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="s">
+        <v>54</v>
+      </c>
+      <c r="B83" t="s">
+        <v>234</v>
+      </c>
+      <c r="C83" t="s">
+        <v>230</v>
+      </c>
+      <c r="D83" s="4"/>
     </row>
   </sheetData>
 </worksheet>
@@ -2946,28 +3196,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>217</v>
+        <v>235</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>218</v>
+        <v>236</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>219</v>
+        <v>237</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>220</v>
+        <v>238</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>221</v>
+        <v>239</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>222</v>
+        <v>240</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>223</v>
+        <v>241</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>224</v>
+        <v>242</v>
       </c>
     </row>
     <row r="2">
@@ -2984,7 +3234,7 @@
         <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>225</v>
+        <v>243</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>15</v>
@@ -2998,10 +3248,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>226</v>
+        <v>244</v>
       </c>
       <c r="B3" t="s">
-        <v>227</v>
+        <v>245</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -3009,10 +3259,10 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>228</v>
+        <v>246</v>
       </c>
       <c r="B4" t="s">
-        <v>229</v>
+        <v>247</v>
       </c>
       <c r="C4" t="s">
         <v>30</v>
@@ -3023,10 +3273,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>230</v>
+        <v>248</v>
       </c>
       <c r="B5" t="s">
-        <v>231</v>
+        <v>249</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -3037,10 +3287,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>232</v>
+        <v>250</v>
       </c>
       <c r="B6" t="s">
-        <v>233</v>
+        <v>251</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -3048,10 +3298,10 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>234</v>
+        <v>252</v>
       </c>
       <c r="B7" t="s">
-        <v>235</v>
+        <v>253</v>
       </c>
       <c r="E7">
         <v>2</v>
@@ -3059,10 +3309,10 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>236</v>
+        <v>254</v>
       </c>
       <c r="B8" t="s">
-        <v>237</v>
+        <v>255</v>
       </c>
       <c r="D8" t="s">
         <v>30</v>
@@ -3073,10 +3323,10 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="B9" t="s">
-        <v>239</v>
+        <v>257</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -3087,10 +3337,10 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>240</v>
+        <v>258</v>
       </c>
       <c r="B10" t="s">
-        <v>241</v>
+        <v>259</v>
       </c>
       <c r="E10">
         <v>0</v>

</xml_diff>

<commit_message>
chore(excelmap): map rokka/suou hooks_config keys to Chinese (Phase 5 followup)
After Phase 5 Excel regen reported 12 warnings (7 rokka + 5 suou keys
without Chinese mappings). Added them across all 4 metadata tables:
- HooksParamMap: 中文名 → JSONKey + 类型
- HooksParamNotes: 给策划看的说明
- HooksParamOrder: 反向 sheet 输出顺序
- CharOrder: 六華 + 蘇芳 加入默认排序末尾

Re-running jsontoexcel now emits zero warnings; xlsx re-regenerated
to pick up the Chinese column labels for both characters' params.
</commit_message>
<xml_diff>
--- a/data/游戏配置表.xlsx
+++ b/data/游戏配置表.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="272">
   <si>
     <t>角色名称</t>
   </si>
@@ -682,46 +682,82 @@
     <t>四印解放后每回合非首次命中时附加的恢复量</t>
   </si>
   <si>
-    <t>adjacent_draw</t>
+    <t>手牌上限</t>
+  </si>
+  <si>
+    <t>六華技能抽牌时的手牌上限（始终生效；仅限技能抽牌路径）</t>
+  </si>
+  <si>
+    <t>触发结算眼数</t>
+  </si>
+  <si>
+    <t>六眼大阵点亮多少眼后触发几何结算（默认 3）</t>
+  </si>
+  <si>
+    <t>等边·回血</t>
+  </si>
+  <si>
+    <t>三眼形成等边三角形 {0,2,4}/{1,3,5} 时回复的生命值</t>
+  </si>
+  <si>
+    <t>等边·摸牌</t>
+  </si>
+  <si>
+    <t>三眼形成等边三角形时额外摸的牌数</t>
+  </si>
+  <si>
+    <t>邻接·摸牌</t>
   </si>
   <si>
     <t>8</t>
   </si>
   <si>
-    <t>hand_size_cap</t>
-  </si>
-  <si>
-    <t>lit_eyes_needed</t>
-  </si>
-  <si>
-    <t>other_damage</t>
-  </si>
-  <si>
-    <t>other_draw</t>
-  </si>
-  <si>
-    <t>triangle_draw</t>
-  </si>
-  <si>
-    <t>triangle_heal</t>
-  </si>
-  <si>
-    <t>fill_base</t>
+    <t>三眼连续相邻（含跨界）时摸的牌数</t>
+  </si>
+  <si>
+    <t>其他·伤害</t>
+  </si>
+  <si>
+    <t>三眼非等边非邻接时对敌方造成的伤害</t>
+  </si>
+  <si>
+    <t>其他·摸牌</t>
+  </si>
+  <si>
+    <t>三眼非等边非邻接时额外摸的牌数</t>
+  </si>
+  <si>
+    <t>基础补牌张数</t>
   </si>
   <si>
     <t>4</t>
   </si>
   <si>
-    <t>revive_synth_draw</t>
-  </si>
-  <si>
-    <t>revive_timeout_sec</t>
-  </si>
-  <si>
-    <t>revive_unsynth_draw</t>
-  </si>
-  <si>
-    <t>skip_cleanup_bonus</t>
+    <t>蘇芳每阶段补牌目标张数（覆盖默认 8）</t>
+  </si>
+  <si>
+    <t>跳过清场后补牌</t>
+  </si>
+  <si>
+    <t>蘇芳本阶段未出攻击牌时，下阶段额外追加抽取的牌数</t>
+  </si>
+  <si>
+    <t>复活倒计时秒数</t>
+  </si>
+  <si>
+    <t>0HP 后复活对话框的总时长，超时则真死亡</t>
+  </si>
+  <si>
+    <t>复活·未合成摸牌</t>
+  </si>
+  <si>
+    <t>拖入两张未合成同色同点牌时复活后摸的牌数</t>
+  </si>
+  <si>
+    <t>复活·已合成摸牌</t>
+  </si>
+  <si>
+    <t>拖入两张已合成同色牌时复活后摸的牌数</t>
   </si>
   <si>
     <t>场地名称</t>
@@ -3040,9 +3076,11 @@
         <v>221</v>
       </c>
       <c r="C71" t="s">
+        <v>125</v>
+      </c>
+      <c r="D71" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="D71" s="4"/>
     </row>
     <row r="72">
       <c r="A72" t="s">
@@ -3052,69 +3090,81 @@
         <v>223</v>
       </c>
       <c r="C72" t="s">
-        <v>125</v>
-      </c>
-      <c r="D72" s="4"/>
+        <v>119</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="s">
         <v>52</v>
       </c>
       <c r="B73" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C73" t="s">
-        <v>119</v>
-      </c>
-      <c r="D73" s="4"/>
+        <v>168</v>
+      </c>
+      <c r="D73" s="4" t="s">
+        <v>226</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="s">
         <v>52</v>
       </c>
       <c r="B74" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C74" t="s">
-        <v>168</v>
-      </c>
-      <c r="D74" s="4"/>
+        <v>119</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="s">
         <v>52</v>
       </c>
       <c r="B75" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="C75" t="s">
-        <v>168</v>
-      </c>
-      <c r="D75" s="4"/>
+        <v>230</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>231</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="s">
         <v>52</v>
       </c>
       <c r="B76" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C76" t="s">
-        <v>119</v>
-      </c>
-      <c r="D76" s="4"/>
+        <v>168</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>233</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="s">
         <v>52</v>
       </c>
       <c r="B77" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="C77" t="s">
         <v>168</v>
       </c>
-      <c r="D77" s="4"/>
+      <c r="D77" s="4" t="s">
+        <v>235</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="3"/>
@@ -3127,60 +3177,70 @@
         <v>54</v>
       </c>
       <c r="B79" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="C79" t="s">
-        <v>230</v>
-      </c>
-      <c r="D79" s="4"/>
+        <v>237</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>238</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="s">
         <v>54</v>
       </c>
       <c r="B80" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="C80" t="s">
-        <v>222</v>
-      </c>
-      <c r="D80" s="4"/>
+        <v>237</v>
+      </c>
+      <c r="D80" s="4" t="s">
+        <v>240</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="s">
         <v>54</v>
       </c>
       <c r="B81" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="C81" t="s">
         <v>125</v>
       </c>
-      <c r="D81" s="4"/>
+      <c r="D81" s="4" t="s">
+        <v>242</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="s">
         <v>54</v>
       </c>
       <c r="B82" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="C82" t="s">
-        <v>230</v>
-      </c>
-      <c r="D82" s="4"/>
+        <v>237</v>
+      </c>
+      <c r="D82" s="4" t="s">
+        <v>244</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="s">
         <v>54</v>
       </c>
       <c r="B83" t="s">
-        <v>234</v>
+        <v>245</v>
       </c>
       <c r="C83" t="s">
         <v>230</v>
       </c>
-      <c r="D83" s="4"/>
+      <c r="D83" s="4" t="s">
+        <v>246</v>
+      </c>
     </row>
   </sheetData>
 </worksheet>
@@ -3196,28 +3256,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2">
@@ -3234,7 +3294,7 @@
         <v>15</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>15</v>
@@ -3248,10 +3308,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="B3" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -3259,10 +3319,10 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="B4" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="C4" t="s">
         <v>30</v>
@@ -3273,10 +3333,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="B5" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -3287,10 +3347,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="B6" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -3298,10 +3358,10 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="B7" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
       <c r="E7">
         <v>2</v>
@@ -3309,10 +3369,10 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="B8" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="D8" t="s">
         <v>30</v>
@@ -3323,10 +3383,10 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="B9" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -3337,10 +3397,10 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="B10" t="s">
-        <v>259</v>
+        <v>271</v>
       </c>
       <c r="E10">
         <v>0</v>

</xml_diff>